<commit_message>
Changes to lib folder gitignore and backend
</commit_message>
<xml_diff>
--- a/Documentos/Documentación/Carta Gantt.xlsx
+++ b/Documentos/Documentación/Carta Gantt.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\ProyectoBibliotecaVirtual\Docs\Documentación\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\Proyecto de titulo Lectura Viva\ProyectoBibliotecaVirtual-main\Documentos\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE8FE468-BF8B-43F6-8956-3020652D117C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD5349F-9719-4390-A55A-171D21D0C75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -586,7 +586,7 @@
       <name val="Roboto"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -800,6 +800,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF002060"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1120,7 +1126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1408,6 +1414,18 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="37" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="36" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="37" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1436,6 +1454,15 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1467,15 +1494,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1808,43 +1826,43 @@
     </row>
     <row r="2" spans="1:93" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="99" t="s">
+      <c r="B2" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="100"/>
-      <c r="D2" s="100"/>
-      <c r="E2" s="100"/>
-      <c r="F2" s="100"/>
-      <c r="G2" s="100"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="102"/>
-      <c r="J2" s="100"/>
-      <c r="K2" s="100"/>
-      <c r="L2" s="100"/>
-      <c r="M2" s="100"/>
-      <c r="N2" s="101"/>
-      <c r="O2" s="103"/>
-      <c r="P2" s="100"/>
-      <c r="Q2" s="100"/>
-      <c r="R2" s="100"/>
-      <c r="S2" s="100"/>
-      <c r="T2" s="100"/>
-      <c r="U2" s="100"/>
-      <c r="V2" s="100"/>
-      <c r="W2" s="100"/>
-      <c r="X2" s="100"/>
-      <c r="Y2" s="100"/>
-      <c r="Z2" s="100"/>
-      <c r="AA2" s="100"/>
-      <c r="AB2" s="100"/>
-      <c r="AC2" s="100"/>
-      <c r="AD2" s="100"/>
-      <c r="AE2" s="100"/>
-      <c r="AF2" s="100"/>
-      <c r="AG2" s="100"/>
-      <c r="AH2" s="100"/>
-      <c r="AI2" s="100"/>
-      <c r="AJ2" s="101"/>
+      <c r="C2" s="104"/>
+      <c r="D2" s="104"/>
+      <c r="E2" s="104"/>
+      <c r="F2" s="104"/>
+      <c r="G2" s="104"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="106"/>
+      <c r="J2" s="104"/>
+      <c r="K2" s="104"/>
+      <c r="L2" s="104"/>
+      <c r="M2" s="104"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="107"/>
+      <c r="P2" s="104"/>
+      <c r="Q2" s="104"/>
+      <c r="R2" s="104"/>
+      <c r="S2" s="104"/>
+      <c r="T2" s="104"/>
+      <c r="U2" s="104"/>
+      <c r="V2" s="104"/>
+      <c r="W2" s="104"/>
+      <c r="X2" s="104"/>
+      <c r="Y2" s="104"/>
+      <c r="Z2" s="104"/>
+      <c r="AA2" s="104"/>
+      <c r="AB2" s="104"/>
+      <c r="AC2" s="104"/>
+      <c r="AD2" s="104"/>
+      <c r="AE2" s="104"/>
+      <c r="AF2" s="104"/>
+      <c r="AG2" s="104"/>
+      <c r="AH2" s="104"/>
+      <c r="AI2" s="104"/>
+      <c r="AJ2" s="105"/>
       <c r="AK2" s="10"/>
       <c r="AL2" s="10"/>
       <c r="AM2" s="1"/>
@@ -2000,39 +2018,39 @@
     </row>
     <row r="4" spans="1:93" ht="21" customHeight="1" x14ac:dyDescent="0.85">
       <c r="A4" s="1"/>
-      <c r="B4" s="104" t="s">
+      <c r="B4" s="108" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="105"/>
-      <c r="D4" s="106" t="s">
+      <c r="C4" s="109"/>
+      <c r="D4" s="110" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="107"/>
-      <c r="F4" s="107"/>
-      <c r="G4" s="108"/>
+      <c r="E4" s="111"/>
+      <c r="F4" s="111"/>
+      <c r="G4" s="112"/>
       <c r="H4" s="15"/>
-      <c r="I4" s="104" t="s">
+      <c r="I4" s="108" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="105"/>
-      <c r="K4" s="105"/>
-      <c r="L4" s="105"/>
-      <c r="M4" s="105"/>
-      <c r="N4" s="105"/>
-      <c r="O4" s="105"/>
-      <c r="P4" s="109"/>
-      <c r="Q4" s="105"/>
-      <c r="R4" s="105"/>
-      <c r="S4" s="105"/>
-      <c r="T4" s="105"/>
-      <c r="U4" s="105"/>
-      <c r="V4" s="105"/>
-      <c r="W4" s="105"/>
-      <c r="X4" s="105"/>
-      <c r="Y4" s="105"/>
-      <c r="Z4" s="105"/>
-      <c r="AA4" s="105"/>
-      <c r="AB4" s="105"/>
+      <c r="J4" s="109"/>
+      <c r="K4" s="109"/>
+      <c r="L4" s="109"/>
+      <c r="M4" s="109"/>
+      <c r="N4" s="109"/>
+      <c r="O4" s="109"/>
+      <c r="P4" s="113"/>
+      <c r="Q4" s="109"/>
+      <c r="R4" s="109"/>
+      <c r="S4" s="109"/>
+      <c r="T4" s="109"/>
+      <c r="U4" s="109"/>
+      <c r="V4" s="109"/>
+      <c r="W4" s="109"/>
+      <c r="X4" s="109"/>
+      <c r="Y4" s="109"/>
+      <c r="Z4" s="109"/>
+      <c r="AA4" s="109"/>
+      <c r="AB4" s="109"/>
       <c r="AC4" s="16"/>
       <c r="AD4" s="9"/>
       <c r="AE4" s="9"/>
@@ -2101,40 +2119,40 @@
     </row>
     <row r="5" spans="1:93" ht="21" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A5" s="1"/>
-      <c r="B5" s="104" t="s">
+      <c r="B5" s="108" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="105"/>
-      <c r="D5" s="118" t="s">
+      <c r="C5" s="109"/>
+      <c r="D5" s="125" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="105"/>
-      <c r="F5" s="105"/>
-      <c r="G5" s="105"/>
+      <c r="E5" s="109"/>
+      <c r="F5" s="109"/>
+      <c r="G5" s="109"/>
       <c r="H5" s="17"/>
-      <c r="I5" s="104" t="s">
+      <c r="I5" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="105"/>
-      <c r="K5" s="105"/>
-      <c r="L5" s="105"/>
-      <c r="M5" s="105"/>
-      <c r="N5" s="105"/>
-      <c r="O5" s="105"/>
-      <c r="P5" s="119">
+      <c r="J5" s="109"/>
+      <c r="K5" s="109"/>
+      <c r="L5" s="109"/>
+      <c r="M5" s="109"/>
+      <c r="N5" s="109"/>
+      <c r="O5" s="109"/>
+      <c r="P5" s="126">
         <v>46106</v>
       </c>
-      <c r="Q5" s="105"/>
-      <c r="R5" s="105"/>
-      <c r="S5" s="105"/>
-      <c r="T5" s="105"/>
-      <c r="U5" s="105"/>
-      <c r="V5" s="105"/>
-      <c r="W5" s="105"/>
-      <c r="X5" s="105"/>
-      <c r="Y5" s="105"/>
-      <c r="Z5" s="105"/>
-      <c r="AA5" s="105"/>
+      <c r="Q5" s="109"/>
+      <c r="R5" s="109"/>
+      <c r="S5" s="109"/>
+      <c r="T5" s="109"/>
+      <c r="U5" s="109"/>
+      <c r="V5" s="109"/>
+      <c r="W5" s="109"/>
+      <c r="X5" s="109"/>
+      <c r="Y5" s="109"/>
+      <c r="Z5" s="109"/>
+      <c r="AA5" s="109"/>
       <c r="AB5" s="18"/>
       <c r="AC5" s="16"/>
       <c r="AD5" s="1"/>
@@ -2394,115 +2412,115 @@
     </row>
     <row r="8" spans="1:93" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="23"/>
-      <c r="B8" s="120" t="s">
+      <c r="B8" s="127" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="120" t="s">
+      <c r="C8" s="127" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="120" t="s">
+      <c r="D8" s="127" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="120" t="s">
+      <c r="E8" s="127" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="120" t="s">
+      <c r="F8" s="127" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="120" t="s">
+      <c r="G8" s="127" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="120" t="s">
+      <c r="H8" s="127" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="117" t="s">
+      <c r="I8" s="124" t="s">
         <v>13</v>
       </c>
-      <c r="J8" s="111"/>
-      <c r="K8" s="111"/>
-      <c r="L8" s="111"/>
-      <c r="M8" s="111"/>
-      <c r="N8" s="111"/>
-      <c r="O8" s="111"/>
-      <c r="P8" s="111"/>
-      <c r="Q8" s="111"/>
-      <c r="R8" s="111"/>
-      <c r="S8" s="111"/>
-      <c r="T8" s="111"/>
-      <c r="U8" s="111"/>
-      <c r="V8" s="111"/>
-      <c r="W8" s="112"/>
-      <c r="X8" s="123" t="s">
+      <c r="J8" s="115"/>
+      <c r="K8" s="115"/>
+      <c r="L8" s="115"/>
+      <c r="M8" s="115"/>
+      <c r="N8" s="115"/>
+      <c r="O8" s="115"/>
+      <c r="P8" s="115"/>
+      <c r="Q8" s="115"/>
+      <c r="R8" s="115"/>
+      <c r="S8" s="115"/>
+      <c r="T8" s="115"/>
+      <c r="U8" s="115"/>
+      <c r="V8" s="115"/>
+      <c r="W8" s="116"/>
+      <c r="X8" s="130" t="s">
         <v>14</v>
       </c>
-      <c r="Y8" s="124"/>
-      <c r="Z8" s="124"/>
-      <c r="AA8" s="124"/>
-      <c r="AB8" s="124"/>
-      <c r="AC8" s="124"/>
-      <c r="AD8" s="124"/>
-      <c r="AE8" s="124"/>
-      <c r="AF8" s="124"/>
-      <c r="AG8" s="124"/>
-      <c r="AH8" s="124"/>
-      <c r="AI8" s="124"/>
-      <c r="AJ8" s="124"/>
-      <c r="AK8" s="124"/>
-      <c r="AL8" s="125"/>
-      <c r="AM8" s="110" t="s">
+      <c r="Y8" s="131"/>
+      <c r="Z8" s="131"/>
+      <c r="AA8" s="131"/>
+      <c r="AB8" s="131"/>
+      <c r="AC8" s="131"/>
+      <c r="AD8" s="131"/>
+      <c r="AE8" s="131"/>
+      <c r="AF8" s="131"/>
+      <c r="AG8" s="131"/>
+      <c r="AH8" s="131"/>
+      <c r="AI8" s="131"/>
+      <c r="AJ8" s="131"/>
+      <c r="AK8" s="131"/>
+      <c r="AL8" s="132"/>
+      <c r="AM8" s="114" t="s">
         <v>15</v>
       </c>
-      <c r="AN8" s="111"/>
-      <c r="AO8" s="111"/>
-      <c r="AP8" s="111"/>
-      <c r="AQ8" s="111"/>
-      <c r="AR8" s="111"/>
-      <c r="AS8" s="111"/>
-      <c r="AT8" s="111"/>
-      <c r="AU8" s="111"/>
-      <c r="AV8" s="111"/>
-      <c r="AW8" s="111"/>
-      <c r="AX8" s="111"/>
-      <c r="AY8" s="111"/>
-      <c r="AZ8" s="111"/>
-      <c r="BA8" s="112"/>
-      <c r="BB8" s="128" t="s">
+      <c r="AN8" s="115"/>
+      <c r="AO8" s="115"/>
+      <c r="AP8" s="115"/>
+      <c r="AQ8" s="115"/>
+      <c r="AR8" s="115"/>
+      <c r="AS8" s="115"/>
+      <c r="AT8" s="115"/>
+      <c r="AU8" s="115"/>
+      <c r="AV8" s="115"/>
+      <c r="AW8" s="115"/>
+      <c r="AX8" s="115"/>
+      <c r="AY8" s="115"/>
+      <c r="AZ8" s="115"/>
+      <c r="BA8" s="116"/>
+      <c r="BB8" s="117" t="s">
         <v>16</v>
       </c>
-      <c r="BC8" s="129"/>
-      <c r="BD8" s="129"/>
-      <c r="BE8" s="129"/>
-      <c r="BF8" s="129"/>
-      <c r="BG8" s="129"/>
-      <c r="BH8" s="129"/>
-      <c r="BI8" s="129"/>
-      <c r="BJ8" s="129"/>
-      <c r="BK8" s="129"/>
-      <c r="BL8" s="129"/>
-      <c r="BM8" s="129"/>
-      <c r="BN8" s="129"/>
-      <c r="BO8" s="129"/>
-      <c r="BP8" s="129"/>
-      <c r="BQ8" s="129"/>
-      <c r="BR8" s="129"/>
-      <c r="BS8" s="129"/>
-      <c r="BT8" s="129"/>
-      <c r="BU8" s="129"/>
-      <c r="BV8" s="129"/>
-      <c r="BW8" s="129"/>
-      <c r="BX8" s="129"/>
-      <c r="BY8" s="129"/>
-      <c r="BZ8" s="129"/>
-      <c r="CA8" s="129"/>
-      <c r="CB8" s="129"/>
-      <c r="CC8" s="129"/>
-      <c r="CD8" s="129"/>
-      <c r="CE8" s="129"/>
-      <c r="CF8" s="129"/>
-      <c r="CG8" s="129"/>
-      <c r="CH8" s="129"/>
-      <c r="CI8" s="129"/>
-      <c r="CJ8" s="130"/>
+      <c r="BC8" s="118"/>
+      <c r="BD8" s="118"/>
+      <c r="BE8" s="118"/>
+      <c r="BF8" s="118"/>
+      <c r="BG8" s="118"/>
+      <c r="BH8" s="118"/>
+      <c r="BI8" s="118"/>
+      <c r="BJ8" s="118"/>
+      <c r="BK8" s="118"/>
+      <c r="BL8" s="118"/>
+      <c r="BM8" s="118"/>
+      <c r="BN8" s="118"/>
+      <c r="BO8" s="118"/>
+      <c r="BP8" s="118"/>
+      <c r="BQ8" s="118"/>
+      <c r="BR8" s="118"/>
+      <c r="BS8" s="118"/>
+      <c r="BT8" s="118"/>
+      <c r="BU8" s="118"/>
+      <c r="BV8" s="118"/>
+      <c r="BW8" s="118"/>
+      <c r="BX8" s="118"/>
+      <c r="BY8" s="118"/>
+      <c r="BZ8" s="118"/>
+      <c r="CA8" s="118"/>
+      <c r="CB8" s="118"/>
+      <c r="CC8" s="118"/>
+      <c r="CD8" s="118"/>
+      <c r="CE8" s="118"/>
+      <c r="CF8" s="118"/>
+      <c r="CG8" s="118"/>
+      <c r="CH8" s="118"/>
+      <c r="CI8" s="118"/>
+      <c r="CJ8" s="119"/>
       <c r="CK8" s="24"/>
       <c r="CL8" s="24"/>
       <c r="CM8" s="24"/>
@@ -2511,142 +2529,142 @@
     </row>
     <row r="9" spans="1:93" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="25"/>
-      <c r="B9" s="121"/>
-      <c r="C9" s="121"/>
-      <c r="D9" s="121"/>
-      <c r="E9" s="121"/>
-      <c r="F9" s="121"/>
-      <c r="G9" s="121"/>
-      <c r="H9" s="121"/>
-      <c r="I9" s="113" t="s">
+      <c r="B9" s="128"/>
+      <c r="C9" s="128"/>
+      <c r="D9" s="128"/>
+      <c r="E9" s="128"/>
+      <c r="F9" s="128"/>
+      <c r="G9" s="128"/>
+      <c r="H9" s="128"/>
+      <c r="I9" s="120" t="s">
         <v>17</v>
       </c>
-      <c r="J9" s="114"/>
-      <c r="K9" s="114"/>
-      <c r="L9" s="114"/>
-      <c r="M9" s="115"/>
-      <c r="N9" s="113" t="s">
+      <c r="J9" s="121"/>
+      <c r="K9" s="121"/>
+      <c r="L9" s="121"/>
+      <c r="M9" s="122"/>
+      <c r="N9" s="120" t="s">
         <v>18</v>
       </c>
-      <c r="O9" s="114"/>
-      <c r="P9" s="114"/>
-      <c r="Q9" s="114"/>
-      <c r="R9" s="115"/>
-      <c r="S9" s="113" t="s">
+      <c r="O9" s="121"/>
+      <c r="P9" s="121"/>
+      <c r="Q9" s="121"/>
+      <c r="R9" s="122"/>
+      <c r="S9" s="120" t="s">
         <v>19</v>
       </c>
-      <c r="T9" s="114"/>
-      <c r="U9" s="114"/>
-      <c r="V9" s="114"/>
-      <c r="W9" s="115"/>
-      <c r="X9" s="126" t="s">
+      <c r="T9" s="121"/>
+      <c r="U9" s="121"/>
+      <c r="V9" s="121"/>
+      <c r="W9" s="122"/>
+      <c r="X9" s="133" t="s">
         <v>20</v>
       </c>
-      <c r="Y9" s="114"/>
-      <c r="Z9" s="114"/>
-      <c r="AA9" s="114"/>
-      <c r="AB9" s="115"/>
-      <c r="AC9" s="126" t="s">
+      <c r="Y9" s="121"/>
+      <c r="Z9" s="121"/>
+      <c r="AA9" s="121"/>
+      <c r="AB9" s="122"/>
+      <c r="AC9" s="133" t="s">
         <v>21</v>
       </c>
-      <c r="AD9" s="114"/>
-      <c r="AE9" s="114"/>
-      <c r="AF9" s="114"/>
-      <c r="AG9" s="115"/>
-      <c r="AH9" s="126" t="s">
+      <c r="AD9" s="121"/>
+      <c r="AE9" s="121"/>
+      <c r="AF9" s="121"/>
+      <c r="AG9" s="122"/>
+      <c r="AH9" s="133" t="s">
         <v>22</v>
       </c>
-      <c r="AI9" s="114"/>
-      <c r="AJ9" s="114"/>
-      <c r="AK9" s="114"/>
-      <c r="AL9" s="115"/>
-      <c r="AM9" s="127" t="s">
+      <c r="AI9" s="121"/>
+      <c r="AJ9" s="121"/>
+      <c r="AK9" s="121"/>
+      <c r="AL9" s="122"/>
+      <c r="AM9" s="134" t="s">
         <v>23</v>
       </c>
-      <c r="AN9" s="114"/>
-      <c r="AO9" s="114"/>
-      <c r="AP9" s="114"/>
-      <c r="AQ9" s="115"/>
-      <c r="AR9" s="127" t="s">
+      <c r="AN9" s="121"/>
+      <c r="AO9" s="121"/>
+      <c r="AP9" s="121"/>
+      <c r="AQ9" s="122"/>
+      <c r="AR9" s="134" t="s">
         <v>24</v>
       </c>
-      <c r="AS9" s="114"/>
-      <c r="AT9" s="114"/>
-      <c r="AU9" s="114"/>
-      <c r="AV9" s="115"/>
-      <c r="AW9" s="127" t="s">
+      <c r="AS9" s="121"/>
+      <c r="AT9" s="121"/>
+      <c r="AU9" s="121"/>
+      <c r="AV9" s="122"/>
+      <c r="AW9" s="134" t="s">
         <v>25</v>
       </c>
-      <c r="AX9" s="114"/>
-      <c r="AY9" s="114"/>
-      <c r="AZ9" s="114"/>
-      <c r="BA9" s="115"/>
-      <c r="BB9" s="116" t="s">
+      <c r="AX9" s="121"/>
+      <c r="AY9" s="121"/>
+      <c r="AZ9" s="121"/>
+      <c r="BA9" s="122"/>
+      <c r="BB9" s="123" t="s">
         <v>26</v>
       </c>
-      <c r="BC9" s="114"/>
-      <c r="BD9" s="114"/>
-      <c r="BE9" s="114"/>
-      <c r="BF9" s="115"/>
-      <c r="BG9" s="116" t="s">
+      <c r="BC9" s="121"/>
+      <c r="BD9" s="121"/>
+      <c r="BE9" s="121"/>
+      <c r="BF9" s="122"/>
+      <c r="BG9" s="123" t="s">
         <v>27</v>
       </c>
-      <c r="BH9" s="114"/>
-      <c r="BI9" s="114"/>
-      <c r="BJ9" s="114"/>
-      <c r="BK9" s="115"/>
-      <c r="BL9" s="116" t="s">
+      <c r="BH9" s="121"/>
+      <c r="BI9" s="121"/>
+      <c r="BJ9" s="121"/>
+      <c r="BK9" s="122"/>
+      <c r="BL9" s="123" t="s">
         <v>28</v>
       </c>
-      <c r="BM9" s="114"/>
-      <c r="BN9" s="114"/>
-      <c r="BO9" s="114"/>
-      <c r="BP9" s="115"/>
-      <c r="BQ9" s="116" t="s">
+      <c r="BM9" s="121"/>
+      <c r="BN9" s="121"/>
+      <c r="BO9" s="121"/>
+      <c r="BP9" s="122"/>
+      <c r="BQ9" s="123" t="s">
         <v>29</v>
       </c>
-      <c r="BR9" s="114"/>
-      <c r="BS9" s="114"/>
-      <c r="BT9" s="114"/>
-      <c r="BU9" s="115"/>
-      <c r="BV9" s="116" t="s">
+      <c r="BR9" s="121"/>
+      <c r="BS9" s="121"/>
+      <c r="BT9" s="121"/>
+      <c r="BU9" s="122"/>
+      <c r="BV9" s="123" t="s">
         <v>30</v>
       </c>
-      <c r="BW9" s="114"/>
-      <c r="BX9" s="114"/>
-      <c r="BY9" s="114"/>
-      <c r="BZ9" s="115"/>
-      <c r="CA9" s="116" t="s">
+      <c r="BW9" s="121"/>
+      <c r="BX9" s="121"/>
+      <c r="BY9" s="121"/>
+      <c r="BZ9" s="122"/>
+      <c r="CA9" s="123" t="s">
         <v>31</v>
       </c>
-      <c r="CB9" s="114"/>
-      <c r="CC9" s="114"/>
-      <c r="CD9" s="114"/>
-      <c r="CE9" s="115"/>
-      <c r="CF9" s="116" t="s">
+      <c r="CB9" s="121"/>
+      <c r="CC9" s="121"/>
+      <c r="CD9" s="121"/>
+      <c r="CE9" s="122"/>
+      <c r="CF9" s="123" t="s">
         <v>32</v>
       </c>
-      <c r="CG9" s="114"/>
-      <c r="CH9" s="114"/>
-      <c r="CI9" s="114"/>
-      <c r="CJ9" s="115"/>
-      <c r="CK9" s="116" t="s">
+      <c r="CG9" s="121"/>
+      <c r="CH9" s="121"/>
+      <c r="CI9" s="121"/>
+      <c r="CJ9" s="122"/>
+      <c r="CK9" s="123" t="s">
         <v>33</v>
       </c>
-      <c r="CL9" s="114"/>
-      <c r="CM9" s="114"/>
-      <c r="CN9" s="114"/>
-      <c r="CO9" s="115"/>
+      <c r="CL9" s="121"/>
+      <c r="CM9" s="121"/>
+      <c r="CN9" s="121"/>
+      <c r="CO9" s="122"/>
     </row>
     <row r="10" spans="1:93" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26"/>
-      <c r="B10" s="122"/>
-      <c r="C10" s="122"/>
-      <c r="D10" s="122"/>
-      <c r="E10" s="122"/>
-      <c r="F10" s="122"/>
-      <c r="G10" s="122"/>
-      <c r="H10" s="122"/>
+      <c r="B10" s="129"/>
+      <c r="C10" s="129"/>
+      <c r="D10" s="129"/>
+      <c r="E10" s="129"/>
+      <c r="F10" s="129"/>
+      <c r="G10" s="129"/>
+      <c r="H10" s="129"/>
       <c r="I10" s="27" t="s">
         <v>34</v>
       </c>
@@ -5306,7 +5324,7 @@
         <v>5</v>
       </c>
       <c r="H33" s="45">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I33" s="53"/>
       <c r="J33" s="56"/>
@@ -5415,7 +5433,7 @@
         <v>5</v>
       </c>
       <c r="H34" s="45">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I34" s="53"/>
       <c r="J34" s="56"/>
@@ -5440,11 +5458,11 @@
       <c r="AC34" s="50"/>
       <c r="AD34" s="50"/>
       <c r="AE34" s="50"/>
-      <c r="AF34" s="50"/>
-      <c r="AG34" s="50"/>
-      <c r="AH34" s="58"/>
-      <c r="AI34" s="58"/>
-      <c r="AJ34" s="58"/>
+      <c r="AF34" s="88"/>
+      <c r="AG34" s="88"/>
+      <c r="AH34" s="99"/>
+      <c r="AI34" s="99"/>
+      <c r="AJ34" s="99"/>
       <c r="AK34" s="58"/>
       <c r="AL34" s="98"/>
       <c r="AM34" s="96"/>
@@ -5524,7 +5542,7 @@
         <v>5</v>
       </c>
       <c r="H35" s="45">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I35" s="53"/>
       <c r="J35" s="56"/>
@@ -5551,11 +5569,11 @@
       <c r="AE35" s="50"/>
       <c r="AF35" s="50"/>
       <c r="AG35" s="50"/>
-      <c r="AH35" s="58"/>
-      <c r="AI35" s="58"/>
-      <c r="AJ35" s="58"/>
-      <c r="AK35" s="58"/>
-      <c r="AL35" s="98"/>
+      <c r="AH35" s="99"/>
+      <c r="AI35" s="99"/>
+      <c r="AJ35" s="99"/>
+      <c r="AK35" s="99"/>
+      <c r="AL35" s="102"/>
       <c r="AM35" s="96"/>
       <c r="AN35" s="58"/>
       <c r="AO35" s="58"/>
@@ -5633,7 +5651,7 @@
         <v>7</v>
       </c>
       <c r="H36" s="45">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="I36" s="70"/>
       <c r="J36" s="71"/>
@@ -5663,9 +5681,9 @@
       <c r="AH36" s="89"/>
       <c r="AI36" s="89"/>
       <c r="AJ36" s="89"/>
-      <c r="AK36" s="58"/>
-      <c r="AL36" s="98"/>
-      <c r="AM36" s="96"/>
+      <c r="AK36" s="89"/>
+      <c r="AL36" s="100"/>
+      <c r="AM36" s="101"/>
       <c r="AN36" s="58"/>
       <c r="AO36" s="58"/>
       <c r="AP36" s="58"/>
@@ -5742,7 +5760,7 @@
         <v>1</v>
       </c>
       <c r="H37" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" s="70"/>
       <c r="J37" s="71"/>
@@ -5774,7 +5792,7 @@
       <c r="AJ37" s="58"/>
       <c r="AK37" s="58"/>
       <c r="AL37" s="98"/>
-      <c r="AM37" s="96"/>
+      <c r="AM37" s="101"/>
       <c r="AN37" s="58"/>
       <c r="AO37" s="58"/>
       <c r="AP37" s="58"/>

</xml_diff>

<commit_message>
feat: unifies management styles and forms, and updates documentation
</commit_message>
<xml_diff>
--- a/Documentos/Documentación/Carta Gantt.xlsx
+++ b/Documentos/Documentación/Carta Gantt.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\Proyecto de titulo Lectura Viva\ProyectoBibliotecaVirtual-main\Documentos\Documentación\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\Proyecto de titulo Lectura Viva\ProyectoBibliotecaVirtual-martin\Documentos\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD5349F-9719-4390-A55A-171D21D0C75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD274558-61A3-481C-8F5C-4B437D2D9EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="124">
   <si>
     <t>Carta Gantt</t>
   </si>
@@ -376,9 +376,6 @@
     <t>4.8</t>
   </si>
   <si>
-    <t>Pruebas QA (Mitigación Riesgos R1-R6)</t>
-  </si>
-  <si>
     <t>Equipo</t>
   </si>
   <si>
@@ -392,6 +389,15 @@
   </si>
   <si>
     <t>Documento Sprint 4 retrospectiva</t>
+  </si>
+  <si>
+    <t>4.11</t>
+  </si>
+  <si>
+    <t>Sistema de compras y carrito</t>
+  </si>
+  <si>
+    <t>Pruebas QA</t>
   </si>
 </sst>
 </file>
@@ -586,7 +592,7 @@
       <name val="Roboto"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="50">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -806,6 +812,78 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF002060"/>
+        <bgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFDE9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor rgb="FFFDE9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FF002060"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor theme="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF002060"/>
+        <bgColor rgb="FFFFF5C9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFFF5C9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1126,7 +1204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="150">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1426,6 +1504,93 @@
     <xf numFmtId="0" fontId="29" fillId="37" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="38" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="39" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="40" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="41" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="42" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="43" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="44" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="45" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="46" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="47" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="48" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1437,10 +1602,6 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1449,51 +1610,13 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="37" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="49" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="45" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1715,7 +1838,7 @@
     <tabColor rgb="FF3D85C6"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:CO1015"/>
+  <dimension ref="A1:CO1016"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.26953125" customWidth="1"/>
@@ -1826,43 +1949,43 @@
     </row>
     <row r="2" spans="1:93" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="103" t="s">
+      <c r="B2" s="138" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="104"/>
-      <c r="D2" s="104"/>
-      <c r="E2" s="104"/>
-      <c r="F2" s="104"/>
-      <c r="G2" s="104"/>
-      <c r="H2" s="105"/>
-      <c r="I2" s="106"/>
-      <c r="J2" s="104"/>
-      <c r="K2" s="104"/>
-      <c r="L2" s="104"/>
-      <c r="M2" s="104"/>
-      <c r="N2" s="105"/>
-      <c r="O2" s="107"/>
-      <c r="P2" s="104"/>
-      <c r="Q2" s="104"/>
-      <c r="R2" s="104"/>
-      <c r="S2" s="104"/>
-      <c r="T2" s="104"/>
-      <c r="U2" s="104"/>
-      <c r="V2" s="104"/>
-      <c r="W2" s="104"/>
-      <c r="X2" s="104"/>
-      <c r="Y2" s="104"/>
-      <c r="Z2" s="104"/>
-      <c r="AA2" s="104"/>
-      <c r="AB2" s="104"/>
-      <c r="AC2" s="104"/>
-      <c r="AD2" s="104"/>
-      <c r="AE2" s="104"/>
-      <c r="AF2" s="104"/>
-      <c r="AG2" s="104"/>
-      <c r="AH2" s="104"/>
-      <c r="AI2" s="104"/>
-      <c r="AJ2" s="105"/>
+      <c r="C2" s="139"/>
+      <c r="D2" s="139"/>
+      <c r="E2" s="139"/>
+      <c r="F2" s="139"/>
+      <c r="G2" s="139"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="141"/>
+      <c r="J2" s="139"/>
+      <c r="K2" s="139"/>
+      <c r="L2" s="139"/>
+      <c r="M2" s="139"/>
+      <c r="N2" s="140"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="139"/>
+      <c r="Q2" s="139"/>
+      <c r="R2" s="139"/>
+      <c r="S2" s="139"/>
+      <c r="T2" s="139"/>
+      <c r="U2" s="139"/>
+      <c r="V2" s="139"/>
+      <c r="W2" s="139"/>
+      <c r="X2" s="139"/>
+      <c r="Y2" s="139"/>
+      <c r="Z2" s="139"/>
+      <c r="AA2" s="139"/>
+      <c r="AB2" s="139"/>
+      <c r="AC2" s="139"/>
+      <c r="AD2" s="139"/>
+      <c r="AE2" s="139"/>
+      <c r="AF2" s="139"/>
+      <c r="AG2" s="139"/>
+      <c r="AH2" s="139"/>
+      <c r="AI2" s="139"/>
+      <c r="AJ2" s="140"/>
       <c r="AK2" s="10"/>
       <c r="AL2" s="10"/>
       <c r="AM2" s="1"/>
@@ -2018,39 +2141,39 @@
     </row>
     <row r="4" spans="1:93" ht="21" customHeight="1" x14ac:dyDescent="0.85">
       <c r="A4" s="1"/>
-      <c r="B4" s="108" t="s">
+      <c r="B4" s="121" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="109"/>
-      <c r="D4" s="110" t="s">
+      <c r="C4" s="122"/>
+      <c r="D4" s="143" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="111"/>
-      <c r="F4" s="111"/>
-      <c r="G4" s="112"/>
+      <c r="E4" s="144"/>
+      <c r="F4" s="144"/>
+      <c r="G4" s="145"/>
       <c r="H4" s="15"/>
-      <c r="I4" s="108" t="s">
+      <c r="I4" s="121" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="109"/>
-      <c r="K4" s="109"/>
-      <c r="L4" s="109"/>
-      <c r="M4" s="109"/>
-      <c r="N4" s="109"/>
-      <c r="O4" s="109"/>
-      <c r="P4" s="113"/>
-      <c r="Q4" s="109"/>
-      <c r="R4" s="109"/>
-      <c r="S4" s="109"/>
-      <c r="T4" s="109"/>
-      <c r="U4" s="109"/>
-      <c r="V4" s="109"/>
-      <c r="W4" s="109"/>
-      <c r="X4" s="109"/>
-      <c r="Y4" s="109"/>
-      <c r="Z4" s="109"/>
-      <c r="AA4" s="109"/>
-      <c r="AB4" s="109"/>
+      <c r="J4" s="122"/>
+      <c r="K4" s="122"/>
+      <c r="L4" s="122"/>
+      <c r="M4" s="122"/>
+      <c r="N4" s="122"/>
+      <c r="O4" s="122"/>
+      <c r="P4" s="146"/>
+      <c r="Q4" s="122"/>
+      <c r="R4" s="122"/>
+      <c r="S4" s="122"/>
+      <c r="T4" s="122"/>
+      <c r="U4" s="122"/>
+      <c r="V4" s="122"/>
+      <c r="W4" s="122"/>
+      <c r="X4" s="122"/>
+      <c r="Y4" s="122"/>
+      <c r="Z4" s="122"/>
+      <c r="AA4" s="122"/>
+      <c r="AB4" s="122"/>
       <c r="AC4" s="16"/>
       <c r="AD4" s="9"/>
       <c r="AE4" s="9"/>
@@ -2119,40 +2242,40 @@
     </row>
     <row r="5" spans="1:93" ht="21" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A5" s="1"/>
-      <c r="B5" s="108" t="s">
+      <c r="B5" s="121" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="109"/>
-      <c r="D5" s="125" t="s">
+      <c r="C5" s="122"/>
+      <c r="D5" s="123" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="109"/>
-      <c r="F5" s="109"/>
-      <c r="G5" s="109"/>
+      <c r="E5" s="122"/>
+      <c r="F5" s="122"/>
+      <c r="G5" s="122"/>
       <c r="H5" s="17"/>
-      <c r="I5" s="108" t="s">
+      <c r="I5" s="121" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="109"/>
-      <c r="K5" s="109"/>
-      <c r="L5" s="109"/>
-      <c r="M5" s="109"/>
-      <c r="N5" s="109"/>
-      <c r="O5" s="109"/>
-      <c r="P5" s="126">
+      <c r="J5" s="122"/>
+      <c r="K5" s="122"/>
+      <c r="L5" s="122"/>
+      <c r="M5" s="122"/>
+      <c r="N5" s="122"/>
+      <c r="O5" s="122"/>
+      <c r="P5" s="124">
         <v>46106</v>
       </c>
-      <c r="Q5" s="109"/>
-      <c r="R5" s="109"/>
-      <c r="S5" s="109"/>
-      <c r="T5" s="109"/>
-      <c r="U5" s="109"/>
-      <c r="V5" s="109"/>
-      <c r="W5" s="109"/>
-      <c r="X5" s="109"/>
-      <c r="Y5" s="109"/>
-      <c r="Z5" s="109"/>
-      <c r="AA5" s="109"/>
+      <c r="Q5" s="122"/>
+      <c r="R5" s="122"/>
+      <c r="S5" s="122"/>
+      <c r="T5" s="122"/>
+      <c r="U5" s="122"/>
+      <c r="V5" s="122"/>
+      <c r="W5" s="122"/>
+      <c r="X5" s="122"/>
+      <c r="Y5" s="122"/>
+      <c r="Z5" s="122"/>
+      <c r="AA5" s="122"/>
       <c r="AB5" s="18"/>
       <c r="AC5" s="16"/>
       <c r="AD5" s="1"/>
@@ -2412,115 +2535,115 @@
     </row>
     <row r="8" spans="1:93" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="23"/>
-      <c r="B8" s="127" t="s">
+      <c r="B8" s="125" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="127" t="s">
+      <c r="C8" s="125" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="127" t="s">
+      <c r="D8" s="125" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="127" t="s">
+      <c r="E8" s="125" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="127" t="s">
+      <c r="F8" s="125" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="127" t="s">
+      <c r="G8" s="125" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="127" t="s">
+      <c r="H8" s="125" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="124" t="s">
+      <c r="I8" s="137" t="s">
         <v>13</v>
       </c>
-      <c r="J8" s="115"/>
-      <c r="K8" s="115"/>
-      <c r="L8" s="115"/>
-      <c r="M8" s="115"/>
-      <c r="N8" s="115"/>
-      <c r="O8" s="115"/>
-      <c r="P8" s="115"/>
-      <c r="Q8" s="115"/>
-      <c r="R8" s="115"/>
-      <c r="S8" s="115"/>
-      <c r="T8" s="115"/>
-      <c r="U8" s="115"/>
-      <c r="V8" s="115"/>
-      <c r="W8" s="116"/>
-      <c r="X8" s="130" t="s">
+      <c r="J8" s="132"/>
+      <c r="K8" s="132"/>
+      <c r="L8" s="132"/>
+      <c r="M8" s="132"/>
+      <c r="N8" s="132"/>
+      <c r="O8" s="132"/>
+      <c r="P8" s="132"/>
+      <c r="Q8" s="132"/>
+      <c r="R8" s="132"/>
+      <c r="S8" s="132"/>
+      <c r="T8" s="132"/>
+      <c r="U8" s="132"/>
+      <c r="V8" s="132"/>
+      <c r="W8" s="133"/>
+      <c r="X8" s="128" t="s">
         <v>14</v>
       </c>
-      <c r="Y8" s="131"/>
-      <c r="Z8" s="131"/>
-      <c r="AA8" s="131"/>
-      <c r="AB8" s="131"/>
-      <c r="AC8" s="131"/>
-      <c r="AD8" s="131"/>
-      <c r="AE8" s="131"/>
-      <c r="AF8" s="131"/>
-      <c r="AG8" s="131"/>
-      <c r="AH8" s="131"/>
-      <c r="AI8" s="131"/>
-      <c r="AJ8" s="131"/>
-      <c r="AK8" s="131"/>
-      <c r="AL8" s="132"/>
-      <c r="AM8" s="114" t="s">
+      <c r="Y8" s="129"/>
+      <c r="Z8" s="129"/>
+      <c r="AA8" s="129"/>
+      <c r="AB8" s="129"/>
+      <c r="AC8" s="129"/>
+      <c r="AD8" s="129"/>
+      <c r="AE8" s="129"/>
+      <c r="AF8" s="129"/>
+      <c r="AG8" s="129"/>
+      <c r="AH8" s="129"/>
+      <c r="AI8" s="129"/>
+      <c r="AJ8" s="129"/>
+      <c r="AK8" s="129"/>
+      <c r="AL8" s="130"/>
+      <c r="AM8" s="131" t="s">
         <v>15</v>
       </c>
-      <c r="AN8" s="115"/>
-      <c r="AO8" s="115"/>
-      <c r="AP8" s="115"/>
-      <c r="AQ8" s="115"/>
-      <c r="AR8" s="115"/>
-      <c r="AS8" s="115"/>
-      <c r="AT8" s="115"/>
-      <c r="AU8" s="115"/>
-      <c r="AV8" s="115"/>
-      <c r="AW8" s="115"/>
-      <c r="AX8" s="115"/>
-      <c r="AY8" s="115"/>
-      <c r="AZ8" s="115"/>
-      <c r="BA8" s="116"/>
-      <c r="BB8" s="117" t="s">
+      <c r="AN8" s="132"/>
+      <c r="AO8" s="132"/>
+      <c r="AP8" s="132"/>
+      <c r="AQ8" s="132"/>
+      <c r="AR8" s="132"/>
+      <c r="AS8" s="132"/>
+      <c r="AT8" s="132"/>
+      <c r="AU8" s="132"/>
+      <c r="AV8" s="132"/>
+      <c r="AW8" s="132"/>
+      <c r="AX8" s="132"/>
+      <c r="AY8" s="132"/>
+      <c r="AZ8" s="132"/>
+      <c r="BA8" s="133"/>
+      <c r="BB8" s="134" t="s">
         <v>16</v>
       </c>
-      <c r="BC8" s="118"/>
-      <c r="BD8" s="118"/>
-      <c r="BE8" s="118"/>
-      <c r="BF8" s="118"/>
-      <c r="BG8" s="118"/>
-      <c r="BH8" s="118"/>
-      <c r="BI8" s="118"/>
-      <c r="BJ8" s="118"/>
-      <c r="BK8" s="118"/>
-      <c r="BL8" s="118"/>
-      <c r="BM8" s="118"/>
-      <c r="BN8" s="118"/>
-      <c r="BO8" s="118"/>
-      <c r="BP8" s="118"/>
-      <c r="BQ8" s="118"/>
-      <c r="BR8" s="118"/>
-      <c r="BS8" s="118"/>
-      <c r="BT8" s="118"/>
-      <c r="BU8" s="118"/>
-      <c r="BV8" s="118"/>
-      <c r="BW8" s="118"/>
-      <c r="BX8" s="118"/>
-      <c r="BY8" s="118"/>
-      <c r="BZ8" s="118"/>
-      <c r="CA8" s="118"/>
-      <c r="CB8" s="118"/>
-      <c r="CC8" s="118"/>
-      <c r="CD8" s="118"/>
-      <c r="CE8" s="118"/>
-      <c r="CF8" s="118"/>
-      <c r="CG8" s="118"/>
-      <c r="CH8" s="118"/>
-      <c r="CI8" s="118"/>
-      <c r="CJ8" s="119"/>
+      <c r="BC8" s="135"/>
+      <c r="BD8" s="135"/>
+      <c r="BE8" s="135"/>
+      <c r="BF8" s="135"/>
+      <c r="BG8" s="135"/>
+      <c r="BH8" s="135"/>
+      <c r="BI8" s="135"/>
+      <c r="BJ8" s="135"/>
+      <c r="BK8" s="135"/>
+      <c r="BL8" s="135"/>
+      <c r="BM8" s="135"/>
+      <c r="BN8" s="135"/>
+      <c r="BO8" s="135"/>
+      <c r="BP8" s="135"/>
+      <c r="BQ8" s="135"/>
+      <c r="BR8" s="135"/>
+      <c r="BS8" s="135"/>
+      <c r="BT8" s="135"/>
+      <c r="BU8" s="135"/>
+      <c r="BV8" s="135"/>
+      <c r="BW8" s="135"/>
+      <c r="BX8" s="135"/>
+      <c r="BY8" s="135"/>
+      <c r="BZ8" s="135"/>
+      <c r="CA8" s="135"/>
+      <c r="CB8" s="135"/>
+      <c r="CC8" s="135"/>
+      <c r="CD8" s="135"/>
+      <c r="CE8" s="135"/>
+      <c r="CF8" s="135"/>
+      <c r="CG8" s="135"/>
+      <c r="CH8" s="135"/>
+      <c r="CI8" s="135"/>
+      <c r="CJ8" s="136"/>
       <c r="CK8" s="24"/>
       <c r="CL8" s="24"/>
       <c r="CM8" s="24"/>
@@ -2529,142 +2652,142 @@
     </row>
     <row r="9" spans="1:93" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="25"/>
-      <c r="B9" s="128"/>
-      <c r="C9" s="128"/>
-      <c r="D9" s="128"/>
-      <c r="E9" s="128"/>
-      <c r="F9" s="128"/>
-      <c r="G9" s="128"/>
-      <c r="H9" s="128"/>
-      <c r="I9" s="120" t="s">
+      <c r="B9" s="126"/>
+      <c r="C9" s="126"/>
+      <c r="D9" s="126"/>
+      <c r="E9" s="126"/>
+      <c r="F9" s="126"/>
+      <c r="G9" s="126"/>
+      <c r="H9" s="126"/>
+      <c r="I9" s="118" t="s">
         <v>17</v>
       </c>
-      <c r="J9" s="121"/>
-      <c r="K9" s="121"/>
-      <c r="L9" s="121"/>
-      <c r="M9" s="122"/>
-      <c r="N9" s="120" t="s">
+      <c r="J9" s="116"/>
+      <c r="K9" s="116"/>
+      <c r="L9" s="116"/>
+      <c r="M9" s="117"/>
+      <c r="N9" s="118" t="s">
         <v>18</v>
       </c>
-      <c r="O9" s="121"/>
-      <c r="P9" s="121"/>
-      <c r="Q9" s="121"/>
-      <c r="R9" s="122"/>
-      <c r="S9" s="120" t="s">
+      <c r="O9" s="116"/>
+      <c r="P9" s="116"/>
+      <c r="Q9" s="116"/>
+      <c r="R9" s="117"/>
+      <c r="S9" s="118" t="s">
         <v>19</v>
       </c>
-      <c r="T9" s="121"/>
-      <c r="U9" s="121"/>
-      <c r="V9" s="121"/>
-      <c r="W9" s="122"/>
-      <c r="X9" s="133" t="s">
+      <c r="T9" s="116"/>
+      <c r="U9" s="116"/>
+      <c r="V9" s="116"/>
+      <c r="W9" s="117"/>
+      <c r="X9" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="Y9" s="121"/>
-      <c r="Z9" s="121"/>
-      <c r="AA9" s="121"/>
-      <c r="AB9" s="122"/>
-      <c r="AC9" s="133" t="s">
+      <c r="Y9" s="116"/>
+      <c r="Z9" s="116"/>
+      <c r="AA9" s="116"/>
+      <c r="AB9" s="117"/>
+      <c r="AC9" s="119" t="s">
         <v>21</v>
       </c>
-      <c r="AD9" s="121"/>
-      <c r="AE9" s="121"/>
-      <c r="AF9" s="121"/>
-      <c r="AG9" s="122"/>
-      <c r="AH9" s="133" t="s">
+      <c r="AD9" s="116"/>
+      <c r="AE9" s="116"/>
+      <c r="AF9" s="116"/>
+      <c r="AG9" s="117"/>
+      <c r="AH9" s="119" t="s">
         <v>22</v>
       </c>
-      <c r="AI9" s="121"/>
-      <c r="AJ9" s="121"/>
-      <c r="AK9" s="121"/>
-      <c r="AL9" s="122"/>
-      <c r="AM9" s="134" t="s">
+      <c r="AI9" s="116"/>
+      <c r="AJ9" s="116"/>
+      <c r="AK9" s="116"/>
+      <c r="AL9" s="117"/>
+      <c r="AM9" s="120" t="s">
         <v>23</v>
       </c>
-      <c r="AN9" s="121"/>
-      <c r="AO9" s="121"/>
-      <c r="AP9" s="121"/>
-      <c r="AQ9" s="122"/>
-      <c r="AR9" s="134" t="s">
+      <c r="AN9" s="116"/>
+      <c r="AO9" s="116"/>
+      <c r="AP9" s="116"/>
+      <c r="AQ9" s="117"/>
+      <c r="AR9" s="120" t="s">
         <v>24</v>
       </c>
-      <c r="AS9" s="121"/>
-      <c r="AT9" s="121"/>
-      <c r="AU9" s="121"/>
-      <c r="AV9" s="122"/>
-      <c r="AW9" s="134" t="s">
+      <c r="AS9" s="116"/>
+      <c r="AT9" s="116"/>
+      <c r="AU9" s="116"/>
+      <c r="AV9" s="117"/>
+      <c r="AW9" s="120" t="s">
         <v>25</v>
       </c>
-      <c r="AX9" s="121"/>
-      <c r="AY9" s="121"/>
-      <c r="AZ9" s="121"/>
-      <c r="BA9" s="122"/>
-      <c r="BB9" s="123" t="s">
+      <c r="AX9" s="116"/>
+      <c r="AY9" s="116"/>
+      <c r="AZ9" s="116"/>
+      <c r="BA9" s="117"/>
+      <c r="BB9" s="115" t="s">
         <v>26</v>
       </c>
-      <c r="BC9" s="121"/>
-      <c r="BD9" s="121"/>
-      <c r="BE9" s="121"/>
-      <c r="BF9" s="122"/>
-      <c r="BG9" s="123" t="s">
+      <c r="BC9" s="116"/>
+      <c r="BD9" s="116"/>
+      <c r="BE9" s="116"/>
+      <c r="BF9" s="117"/>
+      <c r="BG9" s="115" t="s">
         <v>27</v>
       </c>
-      <c r="BH9" s="121"/>
-      <c r="BI9" s="121"/>
-      <c r="BJ9" s="121"/>
-      <c r="BK9" s="122"/>
-      <c r="BL9" s="123" t="s">
+      <c r="BH9" s="116"/>
+      <c r="BI9" s="116"/>
+      <c r="BJ9" s="116"/>
+      <c r="BK9" s="117"/>
+      <c r="BL9" s="115" t="s">
         <v>28</v>
       </c>
-      <c r="BM9" s="121"/>
-      <c r="BN9" s="121"/>
-      <c r="BO9" s="121"/>
-      <c r="BP9" s="122"/>
-      <c r="BQ9" s="123" t="s">
+      <c r="BM9" s="116"/>
+      <c r="BN9" s="116"/>
+      <c r="BO9" s="116"/>
+      <c r="BP9" s="117"/>
+      <c r="BQ9" s="115" t="s">
         <v>29</v>
       </c>
-      <c r="BR9" s="121"/>
-      <c r="BS9" s="121"/>
-      <c r="BT9" s="121"/>
-      <c r="BU9" s="122"/>
-      <c r="BV9" s="123" t="s">
+      <c r="BR9" s="116"/>
+      <c r="BS9" s="116"/>
+      <c r="BT9" s="116"/>
+      <c r="BU9" s="117"/>
+      <c r="BV9" s="115" t="s">
         <v>30</v>
       </c>
-      <c r="BW9" s="121"/>
-      <c r="BX9" s="121"/>
-      <c r="BY9" s="121"/>
-      <c r="BZ9" s="122"/>
-      <c r="CA9" s="123" t="s">
+      <c r="BW9" s="116"/>
+      <c r="BX9" s="116"/>
+      <c r="BY9" s="116"/>
+      <c r="BZ9" s="117"/>
+      <c r="CA9" s="115" t="s">
         <v>31</v>
       </c>
-      <c r="CB9" s="121"/>
-      <c r="CC9" s="121"/>
-      <c r="CD9" s="121"/>
-      <c r="CE9" s="122"/>
-      <c r="CF9" s="123" t="s">
+      <c r="CB9" s="116"/>
+      <c r="CC9" s="116"/>
+      <c r="CD9" s="116"/>
+      <c r="CE9" s="117"/>
+      <c r="CF9" s="115" t="s">
         <v>32</v>
       </c>
-      <c r="CG9" s="121"/>
-      <c r="CH9" s="121"/>
-      <c r="CI9" s="121"/>
-      <c r="CJ9" s="122"/>
-      <c r="CK9" s="123" t="s">
+      <c r="CG9" s="116"/>
+      <c r="CH9" s="116"/>
+      <c r="CI9" s="116"/>
+      <c r="CJ9" s="117"/>
+      <c r="CK9" s="115" t="s">
         <v>33</v>
       </c>
-      <c r="CL9" s="121"/>
-      <c r="CM9" s="121"/>
-      <c r="CN9" s="121"/>
-      <c r="CO9" s="122"/>
+      <c r="CL9" s="116"/>
+      <c r="CM9" s="116"/>
+      <c r="CN9" s="116"/>
+      <c r="CO9" s="117"/>
     </row>
     <row r="10" spans="1:93" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26"/>
-      <c r="B10" s="129"/>
-      <c r="C10" s="129"/>
-      <c r="D10" s="129"/>
-      <c r="E10" s="129"/>
-      <c r="F10" s="129"/>
-      <c r="G10" s="129"/>
-      <c r="H10" s="129"/>
+      <c r="B10" s="127"/>
+      <c r="C10" s="127"/>
+      <c r="D10" s="127"/>
+      <c r="E10" s="127"/>
+      <c r="F10" s="127"/>
+      <c r="G10" s="127"/>
+      <c r="H10" s="127"/>
       <c r="I10" s="27" t="s">
         <v>34</v>
       </c>
@@ -5433,7 +5556,7 @@
         <v>5</v>
       </c>
       <c r="H34" s="45">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I34" s="53"/>
       <c r="J34" s="56"/>
@@ -5542,7 +5665,7 @@
         <v>5</v>
       </c>
       <c r="H35" s="45">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I35" s="53"/>
       <c r="J35" s="56"/>
@@ -5651,7 +5774,7 @@
         <v>7</v>
       </c>
       <c r="H36" s="45">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="I36" s="70"/>
       <c r="J36" s="71"/>
@@ -5860,7 +5983,7 @@
       <c r="E38" s="75"/>
       <c r="F38" s="76"/>
       <c r="G38" s="36">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H38" s="35"/>
       <c r="I38" s="77"/>
@@ -5970,7 +6093,7 @@
         <v>2</v>
       </c>
       <c r="H39" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I39" s="70"/>
       <c r="J39" s="71"/>
@@ -6003,8 +6126,8 @@
       <c r="AK39" s="58"/>
       <c r="AL39" s="98"/>
       <c r="AM39" s="96"/>
-      <c r="AN39" s="58"/>
-      <c r="AO39" s="58"/>
+      <c r="AN39" s="99"/>
+      <c r="AO39" s="99"/>
       <c r="AP39" s="58"/>
       <c r="AQ39" s="58"/>
       <c r="AR39" s="63"/>
@@ -6079,7 +6202,7 @@
         <v>2</v>
       </c>
       <c r="H40" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40" s="53"/>
       <c r="J40" s="56"/>
@@ -6112,8 +6235,8 @@
       <c r="AK40" s="48"/>
       <c r="AL40" s="92"/>
       <c r="AM40" s="90"/>
-      <c r="AN40" s="48"/>
-      <c r="AO40" s="48"/>
+      <c r="AN40" s="83"/>
+      <c r="AO40" s="83"/>
       <c r="AP40" s="48"/>
       <c r="AQ40" s="48"/>
       <c r="AR40" s="51"/>
@@ -6182,13 +6305,13 @@
         <v>46147</v>
       </c>
       <c r="F41" s="43">
-        <v>46167</v>
+        <v>46160</v>
       </c>
       <c r="G41" s="44">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H41" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I41" s="70"/>
       <c r="J41" s="71"/>
@@ -6221,16 +6344,16 @@
       <c r="AK41" s="58"/>
       <c r="AL41" s="98"/>
       <c r="AM41" s="96"/>
-      <c r="AN41" s="58"/>
-      <c r="AO41" s="58"/>
-      <c r="AP41" s="58"/>
-      <c r="AQ41" s="58"/>
-      <c r="AR41" s="63"/>
-      <c r="AS41" s="63"/>
-      <c r="AT41" s="63"/>
-      <c r="AU41" s="63"/>
-      <c r="AV41" s="63"/>
-      <c r="AW41" s="58"/>
+      <c r="AN41" s="99"/>
+      <c r="AO41" s="99"/>
+      <c r="AP41" s="99"/>
+      <c r="AQ41" s="99"/>
+      <c r="AR41" s="103"/>
+      <c r="AS41" s="103"/>
+      <c r="AT41" s="103"/>
+      <c r="AU41" s="103"/>
+      <c r="AV41" s="103"/>
+      <c r="AW41" s="99"/>
       <c r="AX41" s="58"/>
       <c r="AY41" s="58"/>
       <c r="AZ41" s="58"/>
@@ -6297,7 +6420,7 @@
         <v>10</v>
       </c>
       <c r="H42" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I42" s="70"/>
       <c r="J42" s="71"/>
@@ -6331,16 +6454,16 @@
       <c r="AL42" s="98"/>
       <c r="AM42" s="96"/>
       <c r="AN42" s="58"/>
-      <c r="AO42" s="58"/>
-      <c r="AP42" s="58"/>
-      <c r="AQ42" s="58"/>
-      <c r="AR42" s="51"/>
-      <c r="AS42" s="51"/>
-      <c r="AT42" s="51"/>
-      <c r="AU42" s="51"/>
-      <c r="AV42" s="51"/>
-      <c r="AW42" s="58"/>
-      <c r="AX42" s="58"/>
+      <c r="AO42" s="89"/>
+      <c r="AP42" s="89"/>
+      <c r="AQ42" s="89"/>
+      <c r="AR42" s="104"/>
+      <c r="AS42" s="104"/>
+      <c r="AT42" s="104"/>
+      <c r="AU42" s="104"/>
+      <c r="AV42" s="104"/>
+      <c r="AW42" s="89"/>
+      <c r="AX42" s="89"/>
       <c r="AY42" s="58"/>
       <c r="AZ42" s="58"/>
       <c r="BA42" s="98"/>
@@ -6406,7 +6529,7 @@
         <v>10</v>
       </c>
       <c r="H43" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I43" s="70"/>
       <c r="J43" s="71"/>
@@ -6439,16 +6562,16 @@
       <c r="AK43" s="58"/>
       <c r="AL43" s="98"/>
       <c r="AM43" s="96"/>
-      <c r="AN43" s="58"/>
-      <c r="AO43" s="58"/>
-      <c r="AP43" s="58"/>
-      <c r="AQ43" s="58"/>
-      <c r="AR43" s="51"/>
-      <c r="AS43" s="51"/>
-      <c r="AT43" s="51"/>
-      <c r="AU43" s="51"/>
-      <c r="AV43" s="51"/>
-      <c r="AW43" s="58"/>
+      <c r="AN43" s="86"/>
+      <c r="AO43" s="86"/>
+      <c r="AP43" s="86"/>
+      <c r="AQ43" s="86"/>
+      <c r="AR43" s="105"/>
+      <c r="AS43" s="105"/>
+      <c r="AT43" s="105"/>
+      <c r="AU43" s="105"/>
+      <c r="AV43" s="105"/>
+      <c r="AW43" s="86"/>
       <c r="AX43" s="58"/>
       <c r="AY43" s="58"/>
       <c r="AZ43" s="58"/>
@@ -6515,7 +6638,7 @@
         <v>10</v>
       </c>
       <c r="H44" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I44" s="70"/>
       <c r="J44" s="71"/>
@@ -6554,16 +6677,16 @@
       <c r="AQ44" s="58"/>
       <c r="AR44" s="63"/>
       <c r="AS44" s="63"/>
-      <c r="AT44" s="63"/>
-      <c r="AU44" s="63"/>
-      <c r="AV44" s="63"/>
-      <c r="AW44" s="58"/>
-      <c r="AX44" s="58"/>
-      <c r="AY44" s="58"/>
-      <c r="AZ44" s="58"/>
-      <c r="BA44" s="98"/>
-      <c r="BB44" s="96"/>
-      <c r="BC44" s="58"/>
+      <c r="AT44" s="106"/>
+      <c r="AU44" s="106"/>
+      <c r="AV44" s="106"/>
+      <c r="AW44" s="89"/>
+      <c r="AX44" s="89"/>
+      <c r="AY44" s="89"/>
+      <c r="AZ44" s="89"/>
+      <c r="BA44" s="100"/>
+      <c r="BB44" s="101"/>
+      <c r="BC44" s="89"/>
       <c r="BD44" s="58"/>
       <c r="BE44" s="58"/>
       <c r="BF44" s="58"/>
@@ -6618,13 +6741,13 @@
         <v>46148</v>
       </c>
       <c r="F45" s="43">
-        <v>46168</v>
+        <v>46155</v>
       </c>
       <c r="G45" s="44">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="H45" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I45" s="70"/>
       <c r="J45" s="71"/>
@@ -6658,12 +6781,12 @@
       <c r="AL45" s="98"/>
       <c r="AM45" s="96"/>
       <c r="AN45" s="58"/>
-      <c r="AO45" s="58"/>
-      <c r="AP45" s="58"/>
-      <c r="AQ45" s="58"/>
-      <c r="AR45" s="63"/>
-      <c r="AS45" s="63"/>
-      <c r="AT45" s="63"/>
+      <c r="AO45" s="86"/>
+      <c r="AP45" s="86"/>
+      <c r="AQ45" s="86"/>
+      <c r="AR45" s="107"/>
+      <c r="AS45" s="107"/>
+      <c r="AT45" s="107"/>
       <c r="AU45" s="63"/>
       <c r="AV45" s="63"/>
       <c r="AW45" s="58"/>
@@ -6727,13 +6850,13 @@
         <v>46153</v>
       </c>
       <c r="F46" s="43">
-        <v>46164</v>
+        <v>46160</v>
       </c>
       <c r="G46" s="44">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H46" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I46" s="70"/>
       <c r="J46" s="71"/>
@@ -6770,12 +6893,12 @@
       <c r="AO46" s="58"/>
       <c r="AP46" s="58"/>
       <c r="AQ46" s="58"/>
-      <c r="AR46" s="63"/>
-      <c r="AS46" s="63"/>
-      <c r="AT46" s="63"/>
-      <c r="AU46" s="63"/>
-      <c r="AV46" s="63"/>
-      <c r="AW46" s="58"/>
+      <c r="AR46" s="107"/>
+      <c r="AS46" s="107"/>
+      <c r="AT46" s="107"/>
+      <c r="AU46" s="107"/>
+      <c r="AV46" s="107"/>
+      <c r="AW46" s="86"/>
       <c r="AX46" s="58"/>
       <c r="AY46" s="58"/>
       <c r="AZ46" s="58"/>
@@ -6842,7 +6965,7 @@
         <v>1</v>
       </c>
       <c r="H47" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I47" s="70"/>
       <c r="J47" s="71"/>
@@ -6890,7 +7013,7 @@
       <c r="AZ47" s="58"/>
       <c r="BA47" s="98"/>
       <c r="BB47" s="96"/>
-      <c r="BC47" s="58"/>
+      <c r="BC47" s="89"/>
       <c r="BD47" s="58"/>
       <c r="BE47" s="58"/>
       <c r="BF47" s="58"/>
@@ -6942,7 +7065,7 @@
       <c r="E48" s="75"/>
       <c r="F48" s="76"/>
       <c r="G48" s="36">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H48" s="35"/>
       <c r="I48" s="77"/>
@@ -7052,7 +7175,7 @@
         <v>2</v>
       </c>
       <c r="H49" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I49" s="70"/>
       <c r="J49" s="71"/>
@@ -7101,8 +7224,8 @@
       <c r="BA49" s="98"/>
       <c r="BB49" s="96"/>
       <c r="BC49" s="58"/>
-      <c r="BD49" s="58"/>
-      <c r="BE49" s="58"/>
+      <c r="BD49" s="89"/>
+      <c r="BE49" s="89"/>
       <c r="BF49" s="58"/>
       <c r="BG49" s="52"/>
       <c r="BH49" s="52"/>
@@ -7161,7 +7284,7 @@
         <v>2</v>
       </c>
       <c r="H50" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I50" s="53"/>
       <c r="J50" s="56"/>
@@ -7210,8 +7333,8 @@
       <c r="BA50" s="92"/>
       <c r="BB50" s="90"/>
       <c r="BC50" s="48"/>
-      <c r="BD50" s="48"/>
-      <c r="BE50" s="48"/>
+      <c r="BD50" s="109"/>
+      <c r="BE50" s="109"/>
       <c r="BF50" s="48"/>
       <c r="BG50" s="52"/>
       <c r="BH50" s="52"/>
@@ -7270,7 +7393,7 @@
         <v>10</v>
       </c>
       <c r="H51" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I51" s="70"/>
       <c r="J51" s="71"/>
@@ -7322,16 +7445,16 @@
       <c r="BD51" s="58"/>
       <c r="BE51" s="58"/>
       <c r="BF51" s="58"/>
-      <c r="BG51" s="52"/>
-      <c r="BH51" s="52"/>
-      <c r="BI51" s="52"/>
-      <c r="BJ51" s="52"/>
-      <c r="BK51" s="52"/>
-      <c r="BL51" s="58"/>
-      <c r="BM51" s="58"/>
-      <c r="BN51" s="58"/>
-      <c r="BO51" s="58"/>
-      <c r="BP51" s="98"/>
+      <c r="BG51" s="111"/>
+      <c r="BH51" s="111"/>
+      <c r="BI51" s="111"/>
+      <c r="BJ51" s="111"/>
+      <c r="BK51" s="111"/>
+      <c r="BL51" s="99"/>
+      <c r="BM51" s="99"/>
+      <c r="BN51" s="99"/>
+      <c r="BO51" s="99"/>
+      <c r="BP51" s="102"/>
       <c r="BQ51" s="96"/>
       <c r="BR51" s="58"/>
       <c r="BS51" s="58"/>
@@ -7364,22 +7487,22 @@
         <v>107</v>
       </c>
       <c r="C52" s="41" t="s">
-        <v>108</v>
-      </c>
-      <c r="D52" s="55" t="s">
-        <v>44</v>
+        <v>122</v>
+      </c>
+      <c r="D52" s="108" t="s">
+        <v>116</v>
       </c>
       <c r="E52" s="43">
-        <v>46174</v>
+        <v>46171</v>
       </c>
       <c r="F52" s="43">
-        <v>46185</v>
+        <v>46184</v>
       </c>
       <c r="G52" s="44">
         <v>10</v>
       </c>
       <c r="H52" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" s="70"/>
       <c r="J52" s="71"/>
@@ -7430,16 +7553,16 @@
       <c r="BC52" s="58"/>
       <c r="BD52" s="58"/>
       <c r="BE52" s="58"/>
-      <c r="BF52" s="58"/>
-      <c r="BG52" s="64"/>
-      <c r="BH52" s="64"/>
-      <c r="BI52" s="64"/>
-      <c r="BJ52" s="64"/>
-      <c r="BK52" s="64"/>
-      <c r="BL52" s="58"/>
-      <c r="BM52" s="58"/>
-      <c r="BN52" s="58"/>
-      <c r="BO52" s="58"/>
+      <c r="BF52" s="110"/>
+      <c r="BG52" s="112"/>
+      <c r="BH52" s="112"/>
+      <c r="BI52" s="112"/>
+      <c r="BJ52" s="112"/>
+      <c r="BK52" s="112"/>
+      <c r="BL52" s="110"/>
+      <c r="BM52" s="110"/>
+      <c r="BN52" s="110"/>
+      <c r="BO52" s="110"/>
       <c r="BP52" s="98"/>
       <c r="BQ52" s="96"/>
       <c r="BR52" s="58"/>
@@ -7473,22 +7596,22 @@
         <v>109</v>
       </c>
       <c r="C53" s="41" t="s">
-        <v>110</v>
-      </c>
-      <c r="D53" s="42" t="s">
-        <v>41</v>
+        <v>108</v>
+      </c>
+      <c r="D53" s="55" t="s">
+        <v>44</v>
       </c>
       <c r="E53" s="43">
-        <v>46189</v>
+        <v>46174</v>
       </c>
       <c r="F53" s="43">
-        <v>46189</v>
+        <v>46185</v>
       </c>
       <c r="G53" s="44">
+        <v>10</v>
+      </c>
+      <c r="H53" s="45">
         <v>1</v>
-      </c>
-      <c r="H53" s="45">
-        <v>0</v>
       </c>
       <c r="I53" s="70"/>
       <c r="J53" s="71"/>
@@ -7504,7 +7627,7 @@
       <c r="T53" s="58"/>
       <c r="U53" s="58"/>
       <c r="V53" s="58"/>
-      <c r="W53" s="97"/>
+      <c r="W53" s="98"/>
       <c r="X53" s="96"/>
       <c r="Y53" s="58"/>
       <c r="Z53" s="58"/>
@@ -7540,16 +7663,16 @@
       <c r="BD53" s="58"/>
       <c r="BE53" s="58"/>
       <c r="BF53" s="58"/>
-      <c r="BG53" s="64"/>
-      <c r="BH53" s="64"/>
-      <c r="BI53" s="64"/>
-      <c r="BJ53" s="64"/>
-      <c r="BK53" s="64"/>
-      <c r="BL53" s="58"/>
-      <c r="BM53" s="58"/>
-      <c r="BN53" s="58"/>
-      <c r="BO53" s="58"/>
-      <c r="BP53" s="98"/>
+      <c r="BG53" s="113"/>
+      <c r="BH53" s="113"/>
+      <c r="BI53" s="113"/>
+      <c r="BJ53" s="113"/>
+      <c r="BK53" s="113"/>
+      <c r="BL53" s="86"/>
+      <c r="BM53" s="86"/>
+      <c r="BN53" s="86"/>
+      <c r="BO53" s="86"/>
+      <c r="BP53" s="114"/>
       <c r="BQ53" s="96"/>
       <c r="BR53" s="58"/>
       <c r="BS53" s="58"/>
@@ -7582,22 +7705,22 @@
         <v>111</v>
       </c>
       <c r="C54" s="41" t="s">
-        <v>112</v>
-      </c>
-      <c r="D54" s="66" t="s">
-        <v>54</v>
+        <v>110</v>
+      </c>
+      <c r="D54" s="42" t="s">
+        <v>41</v>
       </c>
       <c r="E54" s="43">
-        <v>46190</v>
+        <v>46188</v>
       </c>
       <c r="F54" s="43">
-        <v>46191</v>
+        <v>46188</v>
       </c>
       <c r="G54" s="44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H54" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I54" s="70"/>
       <c r="J54" s="71"/>
@@ -7613,7 +7736,7 @@
       <c r="T54" s="58"/>
       <c r="U54" s="58"/>
       <c r="V54" s="58"/>
-      <c r="W54" s="98"/>
+      <c r="W54" s="97"/>
       <c r="X54" s="96"/>
       <c r="Y54" s="58"/>
       <c r="Z54" s="58"/>
@@ -7649,17 +7772,17 @@
       <c r="BD54" s="58"/>
       <c r="BE54" s="58"/>
       <c r="BF54" s="58"/>
-      <c r="BG54" s="52"/>
-      <c r="BH54" s="52"/>
-      <c r="BI54" s="52"/>
-      <c r="BJ54" s="52"/>
-      <c r="BK54" s="52"/>
+      <c r="BG54" s="64"/>
+      <c r="BH54" s="64"/>
+      <c r="BI54" s="64"/>
+      <c r="BJ54" s="64"/>
+      <c r="BK54" s="64"/>
       <c r="BL54" s="58"/>
       <c r="BM54" s="58"/>
       <c r="BN54" s="58"/>
       <c r="BO54" s="58"/>
       <c r="BP54" s="98"/>
-      <c r="BQ54" s="96"/>
+      <c r="BQ54" s="147"/>
       <c r="BR54" s="58"/>
       <c r="BS54" s="58"/>
       <c r="BT54" s="58"/>
@@ -7691,22 +7814,22 @@
         <v>113</v>
       </c>
       <c r="C55" s="41" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D55" s="66" t="s">
         <v>54</v>
       </c>
       <c r="E55" s="43">
-        <v>46190</v>
+        <v>46188</v>
       </c>
       <c r="F55" s="43">
-        <v>46191</v>
+        <v>46189</v>
       </c>
       <c r="G55" s="44">
         <v>2</v>
       </c>
       <c r="H55" s="45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I55" s="70"/>
       <c r="J55" s="71"/>
@@ -7768,9 +7891,9 @@
       <c r="BN55" s="58"/>
       <c r="BO55" s="58"/>
       <c r="BP55" s="98"/>
-      <c r="BQ55" s="96"/>
-      <c r="BR55" s="58"/>
-      <c r="BS55" s="58"/>
+      <c r="BQ55" s="101"/>
+      <c r="BR55" s="89"/>
+      <c r="BS55" s="148"/>
       <c r="BT55" s="58"/>
       <c r="BU55" s="58"/>
       <c r="BV55" s="52"/>
@@ -7800,24 +7923,24 @@
         <v>115</v>
       </c>
       <c r="C56" s="41" t="s">
-        <v>116</v>
-      </c>
-      <c r="D56" s="80" t="s">
-        <v>117</v>
+        <v>114</v>
+      </c>
+      <c r="D56" s="66" t="s">
+        <v>54</v>
       </c>
       <c r="E56" s="43">
         <v>46188</v>
       </c>
       <c r="F56" s="43">
-        <v>46199</v>
+        <v>46189</v>
       </c>
       <c r="G56" s="44">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H56" s="45">
-        <v>0</v>
-      </c>
-      <c r="I56" s="53"/>
+        <v>1</v>
+      </c>
+      <c r="I56" s="70"/>
       <c r="J56" s="71"/>
       <c r="K56" s="58"/>
       <c r="L56" s="58"/>
@@ -7867,19 +7990,19 @@
       <c r="BD56" s="58"/>
       <c r="BE56" s="58"/>
       <c r="BF56" s="58"/>
-      <c r="BG56" s="64"/>
-      <c r="BH56" s="64"/>
-      <c r="BI56" s="64"/>
-      <c r="BJ56" s="64"/>
-      <c r="BK56" s="64"/>
+      <c r="BG56" s="52"/>
+      <c r="BH56" s="52"/>
+      <c r="BI56" s="52"/>
+      <c r="BJ56" s="52"/>
+      <c r="BK56" s="52"/>
       <c r="BL56" s="58"/>
       <c r="BM56" s="58"/>
       <c r="BN56" s="58"/>
       <c r="BO56" s="58"/>
       <c r="BP56" s="98"/>
-      <c r="BQ56" s="96"/>
-      <c r="BR56" s="58"/>
-      <c r="BS56" s="58"/>
+      <c r="BQ56" s="101"/>
+      <c r="BR56" s="89"/>
+      <c r="BS56" s="148"/>
       <c r="BT56" s="58"/>
       <c r="BU56" s="58"/>
       <c r="BV56" s="52"/>
@@ -7906,25 +8029,25 @@
     <row r="57" spans="1:93" ht="17.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A57" s="39"/>
       <c r="B57" s="40" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C57" s="41" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D57" s="80" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E57" s="43">
+        <v>46188</v>
+      </c>
+      <c r="F57" s="43">
         <v>46199</v>
       </c>
-      <c r="F57" s="43">
-        <v>46213</v>
-      </c>
       <c r="G57" s="44">
-        <v>15</v>
-      </c>
-      <c r="H57" s="59">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="H57" s="45">
+        <v>0.5</v>
       </c>
       <c r="I57" s="53"/>
       <c r="J57" s="71"/>
@@ -7986,16 +8109,16 @@
       <c r="BN57" s="58"/>
       <c r="BO57" s="58"/>
       <c r="BP57" s="98"/>
-      <c r="BQ57" s="96"/>
-      <c r="BR57" s="58"/>
-      <c r="BS57" s="58"/>
-      <c r="BT57" s="58"/>
-      <c r="BU57" s="58"/>
-      <c r="BV57" s="52"/>
-      <c r="BW57" s="52"/>
-      <c r="BX57" s="52"/>
-      <c r="BY57" s="52"/>
-      <c r="BZ57" s="52"/>
+      <c r="BQ57" s="149"/>
+      <c r="BR57" s="110"/>
+      <c r="BS57" s="110"/>
+      <c r="BT57" s="110"/>
+      <c r="BU57" s="110"/>
+      <c r="BV57" s="112"/>
+      <c r="BW57" s="112"/>
+      <c r="BX57" s="112"/>
+      <c r="BY57" s="112"/>
+      <c r="BZ57" s="112"/>
       <c r="CA57" s="58"/>
       <c r="CB57" s="58"/>
       <c r="CC57" s="58"/>
@@ -8015,27 +8138,27 @@
     <row r="58" spans="1:93" ht="17.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A58" s="39"/>
       <c r="B58" s="40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C58" s="41" t="s">
-        <v>121</v>
-      </c>
-      <c r="D58" s="42" t="s">
-        <v>41</v>
+        <v>118</v>
+      </c>
+      <c r="D58" s="80" t="s">
+        <v>116</v>
       </c>
       <c r="E58" s="43">
-        <v>46213</v>
+        <v>46198</v>
       </c>
       <c r="F58" s="43">
-        <v>46213</v>
+        <v>46204</v>
       </c>
       <c r="G58" s="44">
-        <v>1</v>
-      </c>
-      <c r="H58" s="45">
-        <v>0</v>
-      </c>
-      <c r="I58" s="70"/>
+        <v>5</v>
+      </c>
+      <c r="H58" s="59">
+        <v>0.5</v>
+      </c>
+      <c r="I58" s="53"/>
       <c r="J58" s="71"/>
       <c r="K58" s="58"/>
       <c r="L58" s="58"/>
@@ -8049,7 +8172,7 @@
       <c r="T58" s="58"/>
       <c r="U58" s="58"/>
       <c r="V58" s="58"/>
-      <c r="W58" s="97"/>
+      <c r="W58" s="98"/>
       <c r="X58" s="96"/>
       <c r="Y58" s="58"/>
       <c r="Z58" s="58"/>
@@ -8103,11 +8226,11 @@
       <c r="BV58" s="52"/>
       <c r="BW58" s="52"/>
       <c r="BX58" s="52"/>
-      <c r="BY58" s="52"/>
-      <c r="BZ58" s="52"/>
-      <c r="CA58" s="58"/>
-      <c r="CB58" s="58"/>
-      <c r="CC58" s="58"/>
+      <c r="BY58" s="112"/>
+      <c r="BZ58" s="112"/>
+      <c r="CA58" s="110"/>
+      <c r="CB58" s="110"/>
+      <c r="CC58" s="110"/>
       <c r="CD58" s="58"/>
       <c r="CE58" s="98"/>
       <c r="CF58" s="96"/>
@@ -8121,100 +8244,114 @@
       <c r="CN58" s="52"/>
       <c r="CO58" s="52"/>
     </row>
-    <row r="59" spans="1:93" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="20"/>
-      <c r="B59" s="20"/>
-      <c r="C59" s="20"/>
-      <c r="D59" s="20"/>
-      <c r="E59" s="20"/>
-      <c r="F59" s="20"/>
-      <c r="G59" s="81"/>
-      <c r="H59" s="81"/>
-      <c r="I59" s="20"/>
-      <c r="J59" s="20"/>
-      <c r="K59" s="20"/>
-      <c r="L59" s="20"/>
-      <c r="M59" s="20"/>
-      <c r="N59" s="20"/>
-      <c r="O59" s="20"/>
-      <c r="P59" s="20"/>
-      <c r="Q59" s="20"/>
-      <c r="R59" s="20"/>
-      <c r="S59" s="20"/>
-      <c r="T59" s="20"/>
-      <c r="U59" s="20"/>
-      <c r="V59" s="20"/>
-      <c r="W59" s="20"/>
-      <c r="X59" s="20"/>
-      <c r="Y59" s="20"/>
-      <c r="Z59" s="20"/>
-      <c r="AA59" s="20"/>
-      <c r="AB59" s="20"/>
-      <c r="AC59" s="20"/>
-      <c r="AD59" s="20"/>
-      <c r="AE59" s="20"/>
-      <c r="AF59" s="20"/>
-      <c r="AG59" s="20"/>
-      <c r="AH59" s="20"/>
-      <c r="AI59" s="20"/>
-      <c r="AJ59" s="20"/>
-      <c r="AK59" s="20"/>
-      <c r="AL59" s="20"/>
-      <c r="AM59" s="20"/>
-      <c r="AN59" s="20"/>
-      <c r="AO59" s="20"/>
-      <c r="AP59" s="20"/>
-      <c r="AQ59" s="20"/>
-      <c r="AR59" s="20"/>
-      <c r="AS59" s="20"/>
-      <c r="AT59" s="20"/>
-      <c r="AU59" s="20"/>
-      <c r="AV59" s="20"/>
-      <c r="AW59" s="20"/>
-      <c r="AX59" s="20"/>
-      <c r="AY59" s="20"/>
-      <c r="AZ59" s="20"/>
-      <c r="BA59" s="20"/>
-      <c r="BB59" s="20"/>
-      <c r="BC59" s="20"/>
-      <c r="BD59" s="20"/>
-      <c r="BE59" s="20"/>
-      <c r="BF59" s="20"/>
-      <c r="BG59" s="20"/>
-      <c r="BH59" s="20"/>
-      <c r="BI59" s="20"/>
-      <c r="BJ59" s="20"/>
-      <c r="BK59" s="20"/>
-      <c r="BL59" s="20"/>
-      <c r="BM59" s="20"/>
-      <c r="BN59" s="20"/>
-      <c r="BO59" s="20"/>
-      <c r="BP59" s="20"/>
-      <c r="BQ59" s="20"/>
-      <c r="BR59" s="20"/>
-      <c r="BS59" s="20"/>
-      <c r="BT59" s="20"/>
-      <c r="BU59" s="20"/>
-      <c r="BV59" s="20"/>
-      <c r="BW59" s="20"/>
-      <c r="BX59" s="20"/>
-      <c r="BY59" s="20"/>
-      <c r="BZ59" s="20"/>
-      <c r="CA59" s="20"/>
-      <c r="CB59" s="20"/>
-      <c r="CC59" s="20"/>
-      <c r="CD59" s="20"/>
-      <c r="CE59" s="20"/>
-      <c r="CF59" s="20"/>
-      <c r="CG59" s="20"/>
-      <c r="CH59" s="20"/>
-      <c r="CI59" s="20"/>
-      <c r="CJ59" s="20"/>
-      <c r="CK59" s="20"/>
-      <c r="CL59" s="20"/>
-      <c r="CM59" s="20"/>
-      <c r="CN59" s="20"/>
-      <c r="CO59" s="20"/>
+    <row r="59" spans="1:93" ht="17.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="39"/>
+      <c r="B59" s="40" t="s">
+        <v>121</v>
+      </c>
+      <c r="C59" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="D59" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="E59" s="43">
+        <v>46203</v>
+      </c>
+      <c r="F59" s="43">
+        <v>46203</v>
+      </c>
+      <c r="G59" s="44">
+        <v>1</v>
+      </c>
+      <c r="H59" s="45">
+        <v>0.5</v>
+      </c>
+      <c r="I59" s="70"/>
+      <c r="J59" s="71"/>
+      <c r="K59" s="58"/>
+      <c r="L59" s="58"/>
+      <c r="M59" s="58"/>
+      <c r="N59" s="60"/>
+      <c r="O59" s="60"/>
+      <c r="P59" s="60"/>
+      <c r="Q59" s="60"/>
+      <c r="R59" s="60"/>
+      <c r="S59" s="58"/>
+      <c r="T59" s="58"/>
+      <c r="U59" s="58"/>
+      <c r="V59" s="58"/>
+      <c r="W59" s="97"/>
+      <c r="X59" s="96"/>
+      <c r="Y59" s="58"/>
+      <c r="Z59" s="58"/>
+      <c r="AA59" s="58"/>
+      <c r="AB59" s="58"/>
+      <c r="AC59" s="50"/>
+      <c r="AD59" s="50"/>
+      <c r="AE59" s="50"/>
+      <c r="AF59" s="50"/>
+      <c r="AG59" s="50"/>
+      <c r="AH59" s="58"/>
+      <c r="AI59" s="58"/>
+      <c r="AJ59" s="58"/>
+      <c r="AK59" s="58"/>
+      <c r="AL59" s="98"/>
+      <c r="AM59" s="96"/>
+      <c r="AN59" s="58"/>
+      <c r="AO59" s="58"/>
+      <c r="AP59" s="58"/>
+      <c r="AQ59" s="58"/>
+      <c r="AR59" s="63"/>
+      <c r="AS59" s="63"/>
+      <c r="AT59" s="63"/>
+      <c r="AU59" s="63"/>
+      <c r="AV59" s="63"/>
+      <c r="AW59" s="58"/>
+      <c r="AX59" s="58"/>
+      <c r="AY59" s="58"/>
+      <c r="AZ59" s="58"/>
+      <c r="BA59" s="98"/>
+      <c r="BB59" s="96"/>
+      <c r="BC59" s="58"/>
+      <c r="BD59" s="58"/>
+      <c r="BE59" s="58"/>
+      <c r="BF59" s="58"/>
+      <c r="BG59" s="64"/>
+      <c r="BH59" s="64"/>
+      <c r="BI59" s="64"/>
+      <c r="BJ59" s="64"/>
+      <c r="BK59" s="64"/>
+      <c r="BL59" s="58"/>
+      <c r="BM59" s="58"/>
+      <c r="BN59" s="58"/>
+      <c r="BO59" s="58"/>
+      <c r="BP59" s="98"/>
+      <c r="BQ59" s="96"/>
+      <c r="BR59" s="58"/>
+      <c r="BS59" s="58"/>
+      <c r="BT59" s="58"/>
+      <c r="BU59" s="58"/>
+      <c r="BV59" s="52"/>
+      <c r="BW59" s="52"/>
+      <c r="BX59" s="52"/>
+      <c r="BY59" s="52"/>
+      <c r="BZ59" s="52"/>
+      <c r="CA59" s="58"/>
+      <c r="CB59" s="58"/>
+      <c r="CC59" s="58"/>
+      <c r="CD59" s="58"/>
+      <c r="CE59" s="98"/>
+      <c r="CF59" s="96"/>
+      <c r="CG59" s="58"/>
+      <c r="CH59" s="58"/>
+      <c r="CI59" s="58"/>
+      <c r="CJ59" s="58"/>
+      <c r="CK59" s="52"/>
+      <c r="CL59" s="52"/>
+      <c r="CM59" s="52"/>
+      <c r="CN59" s="52"/>
+      <c r="CO59" s="52"/>
     </row>
     <row r="60" spans="1:93" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="20"/>
@@ -8406,7 +8543,101 @@
       <c r="CN61" s="20"/>
       <c r="CO61" s="20"/>
     </row>
-    <row r="62" spans="1:93" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:93" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="20"/>
+      <c r="B62" s="20"/>
+      <c r="C62" s="20"/>
+      <c r="D62" s="20"/>
+      <c r="E62" s="20"/>
+      <c r="F62" s="20"/>
+      <c r="G62" s="81"/>
+      <c r="H62" s="81"/>
+      <c r="I62" s="20"/>
+      <c r="J62" s="20"/>
+      <c r="K62" s="20"/>
+      <c r="L62" s="20"/>
+      <c r="M62" s="20"/>
+      <c r="N62" s="20"/>
+      <c r="O62" s="20"/>
+      <c r="P62" s="20"/>
+      <c r="Q62" s="20"/>
+      <c r="R62" s="20"/>
+      <c r="S62" s="20"/>
+      <c r="T62" s="20"/>
+      <c r="U62" s="20"/>
+      <c r="V62" s="20"/>
+      <c r="W62" s="20"/>
+      <c r="X62" s="20"/>
+      <c r="Y62" s="20"/>
+      <c r="Z62" s="20"/>
+      <c r="AA62" s="20"/>
+      <c r="AB62" s="20"/>
+      <c r="AC62" s="20"/>
+      <c r="AD62" s="20"/>
+      <c r="AE62" s="20"/>
+      <c r="AF62" s="20"/>
+      <c r="AG62" s="20"/>
+      <c r="AH62" s="20"/>
+      <c r="AI62" s="20"/>
+      <c r="AJ62" s="20"/>
+      <c r="AK62" s="20"/>
+      <c r="AL62" s="20"/>
+      <c r="AM62" s="20"/>
+      <c r="AN62" s="20"/>
+      <c r="AO62" s="20"/>
+      <c r="AP62" s="20"/>
+      <c r="AQ62" s="20"/>
+      <c r="AR62" s="20"/>
+      <c r="AS62" s="20"/>
+      <c r="AT62" s="20"/>
+      <c r="AU62" s="20"/>
+      <c r="AV62" s="20"/>
+      <c r="AW62" s="20"/>
+      <c r="AX62" s="20"/>
+      <c r="AY62" s="20"/>
+      <c r="AZ62" s="20"/>
+      <c r="BA62" s="20"/>
+      <c r="BB62" s="20"/>
+      <c r="BC62" s="20"/>
+      <c r="BD62" s="20"/>
+      <c r="BE62" s="20"/>
+      <c r="BF62" s="20"/>
+      <c r="BG62" s="20"/>
+      <c r="BH62" s="20"/>
+      <c r="BI62" s="20"/>
+      <c r="BJ62" s="20"/>
+      <c r="BK62" s="20"/>
+      <c r="BL62" s="20"/>
+      <c r="BM62" s="20"/>
+      <c r="BN62" s="20"/>
+      <c r="BO62" s="20"/>
+      <c r="BP62" s="20"/>
+      <c r="BQ62" s="20"/>
+      <c r="BR62" s="20"/>
+      <c r="BS62" s="20"/>
+      <c r="BT62" s="20"/>
+      <c r="BU62" s="20"/>
+      <c r="BV62" s="20"/>
+      <c r="BW62" s="20"/>
+      <c r="BX62" s="20"/>
+      <c r="BY62" s="20"/>
+      <c r="BZ62" s="20"/>
+      <c r="CA62" s="20"/>
+      <c r="CB62" s="20"/>
+      <c r="CC62" s="20"/>
+      <c r="CD62" s="20"/>
+      <c r="CE62" s="20"/>
+      <c r="CF62" s="20"/>
+      <c r="CG62" s="20"/>
+      <c r="CH62" s="20"/>
+      <c r="CI62" s="20"/>
+      <c r="CJ62" s="20"/>
+      <c r="CK62" s="20"/>
+      <c r="CL62" s="20"/>
+      <c r="CM62" s="20"/>
+      <c r="CN62" s="20"/>
+      <c r="CO62" s="20"/>
+    </row>
     <row r="63" spans="1:93" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="64" spans="1:93" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -9360,16 +9591,28 @@
     <row r="1013" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1014" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1015" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1016" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="CK9:CO9"/>
-    <mergeCell ref="S9:W9"/>
-    <mergeCell ref="X9:AB9"/>
-    <mergeCell ref="AC9:AG9"/>
-    <mergeCell ref="AH9:AL9"/>
-    <mergeCell ref="AM9:AQ9"/>
-    <mergeCell ref="AR9:AV9"/>
-    <mergeCell ref="AW9:BA9"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="I2:N2"/>
+    <mergeCell ref="O2:AJ2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="I4:O4"/>
+    <mergeCell ref="P4:AB4"/>
+    <mergeCell ref="AM8:BA8"/>
+    <mergeCell ref="BB8:CJ8"/>
+    <mergeCell ref="I9:M9"/>
+    <mergeCell ref="N9:R9"/>
+    <mergeCell ref="BB9:BF9"/>
+    <mergeCell ref="BG9:BK9"/>
+    <mergeCell ref="BL9:BP9"/>
+    <mergeCell ref="BQ9:BU9"/>
+    <mergeCell ref="BV9:BZ9"/>
+    <mergeCell ref="CA9:CE9"/>
+    <mergeCell ref="CF9:CJ9"/>
+    <mergeCell ref="I8:W8"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D5:G5"/>
     <mergeCell ref="I5:O5"/>
@@ -9382,25 +9625,14 @@
     <mergeCell ref="F8:F10"/>
     <mergeCell ref="G8:G10"/>
     <mergeCell ref="H8:H10"/>
-    <mergeCell ref="AM8:BA8"/>
-    <mergeCell ref="BB8:CJ8"/>
-    <mergeCell ref="I9:M9"/>
-    <mergeCell ref="N9:R9"/>
-    <mergeCell ref="BB9:BF9"/>
-    <mergeCell ref="BG9:BK9"/>
-    <mergeCell ref="BL9:BP9"/>
-    <mergeCell ref="BQ9:BU9"/>
-    <mergeCell ref="BV9:BZ9"/>
-    <mergeCell ref="CA9:CE9"/>
-    <mergeCell ref="CF9:CJ9"/>
-    <mergeCell ref="I8:W8"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="I2:N2"/>
-    <mergeCell ref="O2:AJ2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:G4"/>
-    <mergeCell ref="I4:O4"/>
-    <mergeCell ref="P4:AB4"/>
+    <mergeCell ref="CK9:CO9"/>
+    <mergeCell ref="S9:W9"/>
+    <mergeCell ref="X9:AB9"/>
+    <mergeCell ref="AC9:AG9"/>
+    <mergeCell ref="AH9:AL9"/>
+    <mergeCell ref="AM9:AQ9"/>
+    <mergeCell ref="AR9:AV9"/>
+    <mergeCell ref="AW9:BA9"/>
   </mergeCells>
   <conditionalFormatting sqref="H12:H26 H29 H40 H50">
     <cfRule type="colorScale" priority="1">
@@ -9420,7 +9652,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H28:H37 H18 H39:H58">
+  <conditionalFormatting sqref="H28:H37 H18 H39:H59">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>